<commit_message>
Sync goods catalog from Excel and route inquiries to m3auto.lk@gmail.com.
</commit_message>
<xml_diff>
--- a/resources/Goods and Services list.xlsx
+++ b/resources/Goods and Services list.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sahan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sahan\Desktop\Other\Projects\M3 Auto Website\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25DF49EF-D957-462C-9DDA-A0F26036EA93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACC972D4-1FB9-4E62-98C4-5A8AB2128A70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="203">
   <si>
     <t>Category</t>
   </si>
@@ -482,9 +482,6 @@
     <t>VALVOLINE 880911 - 15W-40 / 5L DIESEL MOTOR OIL</t>
   </si>
   <si>
-    <t>VALVOLINE 881097 - 15W-40 / 1L FREE</t>
-  </si>
-  <si>
     <t>VALVOLINE 881097 - 15W-40 / 1L DIESEL MOTOR OIL</t>
   </si>
   <si>
@@ -630,36 +627,6 @@
   </si>
   <si>
     <t>WURTH DOT - 4 BREAK FLUID 500ML</t>
-  </si>
-  <si>
-    <t>AIR FRESHNER</t>
-  </si>
-  <si>
-    <t>DASH</t>
-  </si>
-  <si>
-    <t>RAIHAN COOL ICE / 40G</t>
-  </si>
-  <si>
-    <t>DASH AIR FRESHNER - GEL TRAY / 40G</t>
-  </si>
-  <si>
-    <t>DASH AIR POCKET / 10G</t>
-  </si>
-  <si>
-    <t>DASH A.F. GEL POCKET - PURE FAST / 10G</t>
-  </si>
-  <si>
-    <t>DASH AIR FRESHNER SPRAY BOTTLE / 500ML</t>
-  </si>
-  <si>
-    <t>TISSUE BOX</t>
-  </si>
-  <si>
-    <t>MINT</t>
-  </si>
-  <si>
-    <t>MINT FACIAL TISSUE 1 BOX</t>
   </si>
   <si>
     <t>CAR SCANNING</t>
@@ -981,7 +948,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:V1012"/>
+  <dimension ref="A1:V1011"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.44140625" customWidth="1"/>
@@ -1653,16 +1620,16 @@
     </row>
     <row r="86" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A86" s="3"/>
-      <c r="B86" s="3"/>
+      <c r="B86" s="3" t="s">
+        <v>164</v>
+      </c>
       <c r="C86" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A87" s="3"/>
-      <c r="B87" s="3" t="s">
-        <v>165</v>
-      </c>
+      <c r="B87" s="3"/>
       <c r="C87" s="6" t="s">
         <v>166</v>
       </c>
@@ -1704,16 +1671,16 @@
     </row>
     <row r="93" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A93" s="3"/>
-      <c r="B93" s="3"/>
+      <c r="B93" s="3" t="s">
+        <v>172</v>
+      </c>
       <c r="C93" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="94" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A94" s="3"/>
-      <c r="B94" s="3" t="s">
-        <v>173</v>
-      </c>
+      <c r="B94" s="3"/>
       <c r="C94" s="6" t="s">
         <v>174</v>
       </c>
@@ -1762,27 +1729,27 @@
     </row>
     <row r="101" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A101" s="3"/>
-      <c r="B101" s="3"/>
+      <c r="B101" s="3" t="s">
+        <v>181</v>
+      </c>
       <c r="C101" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="102" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A102" s="3"/>
+      <c r="A102" s="3" t="s">
+        <v>183</v>
+      </c>
       <c r="B102" s="3" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C102" s="6" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="103" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A103" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="B103" s="3" t="s">
-        <v>185</v>
-      </c>
+      <c r="A103" s="3"/>
+      <c r="B103" s="3"/>
       <c r="C103" s="6" t="s">
         <v>186</v>
       </c>
@@ -1824,16 +1791,16 @@
     </row>
     <row r="109" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A109" s="3"/>
-      <c r="B109" s="3"/>
+      <c r="B109" s="3" t="s">
+        <v>134</v>
+      </c>
       <c r="C109" s="6" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="110" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A110" s="3"/>
-      <c r="B110" s="3" t="s">
-        <v>134</v>
-      </c>
+      <c r="B110" s="3"/>
       <c r="C110" s="6" t="s">
         <v>193</v>
       </c>
@@ -1897,59 +1864,37 @@
     <row r="119" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A119" s="3"/>
       <c r="B119" s="3"/>
-      <c r="C119" s="6" t="s">
-        <v>202</v>
-      </c>
+      <c r="C119" s="6"/>
     </row>
     <row r="120" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A120" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="B120" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="C120" s="6" t="s">
-        <v>205</v>
-      </c>
+      <c r="A120" s="3"/>
+      <c r="B120" s="3"/>
+      <c r="C120" s="6"/>
     </row>
     <row r="121" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A121" s="3"/>
       <c r="B121" s="3"/>
-      <c r="C121" s="6" t="s">
-        <v>206</v>
-      </c>
+      <c r="C121" s="6"/>
     </row>
     <row r="122" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A122" s="3"/>
       <c r="B122" s="3"/>
-      <c r="C122" s="6" t="s">
-        <v>207</v>
-      </c>
+      <c r="C122" s="6"/>
     </row>
     <row r="123" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A123" s="3"/>
       <c r="B123" s="3"/>
-      <c r="C123" s="6" t="s">
-        <v>208</v>
-      </c>
+      <c r="C123" s="6"/>
     </row>
     <row r="124" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A124" s="3"/>
       <c r="B124" s="3"/>
-      <c r="C124" s="6" t="s">
-        <v>209</v>
-      </c>
+      <c r="C124" s="6"/>
     </row>
     <row r="125" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A125" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B125" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="C125" s="6" t="s">
-        <v>212</v>
-      </c>
+      <c r="A125" s="3"/>
+      <c r="B125" s="3"/>
+      <c r="C125" s="6"/>
     </row>
     <row r="126" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A126" s="3"/>
@@ -1987,9 +1932,7 @@
       <c r="C132" s="6"/>
     </row>
     <row r="133" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A133" s="3"/>
-      <c r="B133" s="3"/>
-      <c r="C133" s="6"/>
+      <c r="C133" s="7"/>
     </row>
     <row r="134" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="C134" s="7"/>
@@ -4624,9 +4567,6 @@
     </row>
     <row r="1011" spans="3:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="C1011" s="7"/>
-    </row>
-    <row r="1012" spans="3:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="C1012" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5008,13 +4948,13 @@
     </row>
     <row r="45" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update service category images and sync services from Excel.
Map each workshop category to its dedicated photo and refresh catalog content.
</commit_message>
<xml_diff>
--- a/resources/Goods and Services list.xlsx
+++ b/resources/Goods and Services list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sahan\Desktop\Other\Projects\M3 Auto Website\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACC972D4-1FB9-4E62-98C4-5A8AB2128A70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E509CFB2-E8E9-4CBF-BABC-E91791376440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Goods" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="199">
   <si>
     <t>Category</t>
   </si>
@@ -233,24 +233,15 @@
     <t>EXTERIOR</t>
   </si>
   <si>
-    <t xml:space="preserve">FULL BIKE WASH </t>
-  </si>
-  <si>
     <t>SUZUKI AIR FILTER 13780 - 74M00</t>
   </si>
   <si>
     <t>FULL BIKE WASH WITH WAXING</t>
   </si>
   <si>
-    <t>BIKE CHAIN REGREASING</t>
-  </si>
-  <si>
     <t>CAR BODY WASH</t>
   </si>
   <si>
-    <t>SUV BODY WASH</t>
-  </si>
-  <si>
     <t>SUZUKI AIR FILTER 13780 - 80GA0</t>
   </si>
   <si>
@@ -273,9 +264,6 @@
   </si>
   <si>
     <t>SUZUKI AIR FILTER 13780 - 59500</t>
-  </si>
-  <si>
-    <t>SUV EXTERIOR BODY WAXING</t>
   </si>
   <si>
     <t>CAR DETAILING</t>
@@ -1094,173 +1082,173 @@
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="6" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="6" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="6" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="6" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="6" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="6" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="3" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="6" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="6" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="6" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="6" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="6" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>17</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="6" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="6" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
@@ -1269,99 +1257,99 @@
         <v>63</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="6" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="6" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
       <c r="B43" s="3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="6" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="6" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>17</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="6" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="6" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="6" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="6" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="6" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
@@ -1370,495 +1358,495 @@
         <v>63</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A54" s="3"/>
       <c r="B54" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="6" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="6" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A57" s="3"/>
       <c r="B57" s="3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
       <c r="B58" s="3" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="6" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="6" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="C62" s="6" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
       <c r="C63" s="6" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="6" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="6" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="6" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="6" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
       <c r="C68" s="6" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="6" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="6" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
       <c r="C71" s="6" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="6" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
       <c r="C73" s="6" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
       <c r="C75" s="6" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="6" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="77" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
       <c r="C77" s="6" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="C78" s="6" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="79" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="C79" s="6" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="80" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
       <c r="C80" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
       <c r="C81" s="6" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="82" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
       <c r="C82" s="6" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="83" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="6" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="84" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
       <c r="C84" s="6" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A85" s="3"/>
       <c r="B85" s="3"/>
       <c r="C85" s="6" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="86" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A86" s="3"/>
       <c r="B86" s="3" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="6" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
     </row>
     <row r="88" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
       <c r="C88" s="6" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="89" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
       <c r="C89" s="6" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="90" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
       <c r="C90" s="6" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="91" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
       <c r="C91" s="6" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="92" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
       <c r="C92" s="6" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="93" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A93" s="3"/>
       <c r="B93" s="3" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="94" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
       <c r="C94" s="6" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="95" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A95" s="3"/>
       <c r="B95" s="3"/>
       <c r="C95" s="6" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="96" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
       <c r="C96" s="6" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="97" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
       <c r="C97" s="6" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="98" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
       <c r="C98" s="6" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="99" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
       <c r="C99" s="6" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="100" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
       <c r="C100" s="6" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A101" s="3"/>
       <c r="B101" s="3" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C101" s="6" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="102" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C102" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="103" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
       <c r="C103" s="6" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="104" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A104" s="3"/>
       <c r="B104" s="3"/>
       <c r="C104" s="6" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="105" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A105" s="3"/>
       <c r="B105" s="3"/>
       <c r="C105" s="6" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="106" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A106" s="3"/>
       <c r="B106" s="3"/>
       <c r="C106" s="6" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
     </row>
     <row r="107" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A107" s="3"/>
       <c r="B107" s="3"/>
       <c r="C107" s="6" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="108" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A108" s="3"/>
       <c r="B108" s="3"/>
       <c r="C108" s="6" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="109" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A109" s="3"/>
       <c r="B109" s="3" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C109" s="6" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
     <row r="110" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A110" s="3"/>
       <c r="B110" s="3"/>
       <c r="C110" s="6" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="111" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A111" s="3"/>
       <c r="B111" s="3"/>
       <c r="C111" s="6" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="112" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A112" s="3"/>
       <c r="B112" s="3"/>
       <c r="C112" s="6" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="113" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A113" s="3"/>
       <c r="B113" s="3"/>
       <c r="C113" s="6" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
     </row>
     <row r="114" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A114" s="3"/>
       <c r="B114" s="3"/>
       <c r="C114" s="6" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="115" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A115" s="3"/>
       <c r="B115" s="3"/>
       <c r="C115" s="6" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="116" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A116" s="3"/>
       <c r="B116" s="3"/>
       <c r="C116" s="6" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="117" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A117" s="3"/>
       <c r="B117" s="3"/>
       <c r="C117" s="6" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="118" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A118" s="3"/>
       <c r="B118" s="3"/>
       <c r="C118" s="6" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="119" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
@@ -4578,7 +4566,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.44140625" customWidth="1"/>
@@ -4862,7 +4850,7 @@
         <v>69</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
@@ -4876,86 +4864,78 @@
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A39" s="3"/>
-      <c r="B39" s="3"/>
+      <c r="A39" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>81</v>
+      </c>
       <c r="C39" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A41" s="3"/>
-      <c r="B41" s="3"/>
+      <c r="A41" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>198</v>
+      </c>
       <c r="C41" s="3" t="s">
-        <v>82</v>
+        <v>198</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
-      <c r="C42" s="3" t="s">
-        <v>84</v>
-      </c>
+      <c r="C42" s="3"/>
     </row>
     <row r="43" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A43" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>86</v>
-      </c>
+      <c r="A43" s="3"/>
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
     </row>
     <row r="44" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
-      <c r="C44" s="3" t="s">
-        <v>88</v>
-      </c>
+      <c r="C44" s="3"/>
     </row>
     <row r="45" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>202</v>
-      </c>
+      <c r="A45" s="3"/>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
     </row>
     <row r="46" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A46" s="3"/>
@@ -5212,26 +5192,6 @@
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
     </row>
-    <row r="97" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A97" s="3"/>
-      <c r="B97" s="3"/>
-      <c r="C97" s="3"/>
-    </row>
-    <row r="98" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A98" s="3"/>
-      <c r="B98" s="3"/>
-      <c r="C98" s="3"/>
-    </row>
-    <row r="99" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A99" s="3"/>
-      <c r="B99" s="3"/>
-      <c r="C99" s="3"/>
-    </row>
-    <row r="100" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A100" s="3"/>
-      <c r="B100" s="3"/>
-      <c r="C100" s="3"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>